<commit_message>
Update kode Material Part: 28.08.2026
</commit_message>
<xml_diff>
--- a/BOM/Use.xlsx
+++ b/BOM/Use.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DANIEL\ANTIGRAVITY\PROJEK\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F9295F5-5597-4309-9C82-711C983F3E35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A287FB8-347A-4303-BC8F-717E110EE736}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{50E5FA24-8F04-4F2F-94DC-6D079599AFC2}"/>
+    <workbookView xWindow="-20775" yWindow="3240" windowWidth="14400" windowHeight="7275" xr2:uid="{50E5FA24-8F04-4F2F-94DC-6D079599AFC2}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="484" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="485" uniqueCount="104">
   <si>
     <t>No.</t>
   </si>
@@ -343,6 +343,9 @@
   </si>
   <si>
     <t>LLL</t>
+  </si>
+  <si>
+    <t>P Sloc</t>
   </si>
 </sst>
 </file>
@@ -600,6 +603,9 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -622,9 +628,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="166" fontId="4" fillId="2" borderId="2" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -974,7 +977,7 @@
     <col min="28" max="28" width="10.08984375" bestFit="1" customWidth="1"/>
     <col min="29" max="31" width="6.81640625" customWidth="1"/>
     <col min="32" max="32" width="14.36328125" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="5.36328125" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="7.08984375" bestFit="1" customWidth="1"/>
     <col min="34" max="34" width="19.08984375" bestFit="1" customWidth="1"/>
     <col min="35" max="35" width="21.26953125" bestFit="1" customWidth="1"/>
   </cols>
@@ -1018,49 +1021,51 @@
       <c r="R1" s="32" t="s">
         <v>9</v>
       </c>
-      <c r="S1" s="35" t="s">
+      <c r="S1" s="36" t="s">
         <v>10</v>
       </c>
-      <c r="T1" s="36" t="s">
+      <c r="T1" s="37" t="s">
         <v>11</v>
       </c>
-      <c r="U1" s="37" t="s">
+      <c r="U1" s="38" t="s">
         <v>12</v>
       </c>
-      <c r="V1" s="38" t="s">
+      <c r="V1" s="39" t="s">
         <v>13</v>
       </c>
-      <c r="W1" s="39" t="s">
+      <c r="W1" s="40" t="s">
         <v>14</v>
       </c>
-      <c r="X1" s="39" t="s">
+      <c r="X1" s="40" t="s">
         <v>15</v>
       </c>
-      <c r="Y1" s="37" t="s">
-        <v>16</v>
-      </c>
-      <c r="Z1" s="37" t="s">
+      <c r="Y1" s="38" t="s">
+        <v>16</v>
+      </c>
+      <c r="Z1" s="38" t="s">
         <v>17</v>
       </c>
-      <c r="AA1" s="40" t="s">
+      <c r="AA1" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="AB1" s="40" t="s">
+      <c r="AB1" s="41" t="s">
         <v>19</v>
       </c>
-      <c r="AC1" s="33" t="s">
+      <c r="AC1" s="34" t="s">
         <v>20</v>
       </c>
-      <c r="AD1" s="33"/>
-      <c r="AE1" s="33"/>
-      <c r="AF1" s="33" t="s">
+      <c r="AD1" s="34"/>
+      <c r="AE1" s="34"/>
+      <c r="AF1" s="34" t="s">
         <v>21</v>
       </c>
-      <c r="AG1" s="33"/>
-      <c r="AH1" s="34" t="s">
+      <c r="AG1" s="34" t="s">
+        <v>103</v>
+      </c>
+      <c r="AH1" s="35" t="s">
         <v>22</v>
       </c>
-      <c r="AI1" s="34" t="s">
+      <c r="AI1" s="35" t="s">
         <v>23</v>
       </c>
     </row>
@@ -1068,18 +1073,18 @@
       <c r="A2" s="32"/>
       <c r="B2" s="32"/>
       <c r="C2" s="32"/>
-      <c r="D2" s="41" t="s">
+      <c r="D2" s="33" t="s">
         <v>24</v>
       </c>
-      <c r="E2" s="41"/>
-      <c r="F2" s="41" t="s">
+      <c r="E2" s="33"/>
+      <c r="F2" s="33" t="s">
         <v>25</v>
       </c>
-      <c r="G2" s="41"/>
-      <c r="H2" s="41" t="s">
+      <c r="G2" s="33"/>
+      <c r="H2" s="33" t="s">
         <v>26</v>
       </c>
-      <c r="I2" s="41"/>
+      <c r="I2" s="33"/>
       <c r="J2" s="29"/>
       <c r="K2" s="30" t="s">
         <v>24</v>
@@ -1095,23 +1100,23 @@
       <c r="P2" s="32"/>
       <c r="Q2" s="32"/>
       <c r="R2" s="32"/>
-      <c r="S2" s="35"/>
-      <c r="T2" s="36"/>
-      <c r="U2" s="37"/>
-      <c r="V2" s="38"/>
-      <c r="W2" s="39"/>
-      <c r="X2" s="39"/>
-      <c r="Y2" s="37"/>
-      <c r="Z2" s="37"/>
-      <c r="AA2" s="40"/>
-      <c r="AB2" s="40"/>
-      <c r="AC2" s="33"/>
-      <c r="AD2" s="33"/>
-      <c r="AE2" s="33"/>
-      <c r="AF2" s="33"/>
-      <c r="AG2" s="33"/>
-      <c r="AH2" s="34"/>
-      <c r="AI2" s="34"/>
+      <c r="S2" s="36"/>
+      <c r="T2" s="37"/>
+      <c r="U2" s="38"/>
+      <c r="V2" s="39"/>
+      <c r="W2" s="40"/>
+      <c r="X2" s="40"/>
+      <c r="Y2" s="38"/>
+      <c r="Z2" s="38"/>
+      <c r="AA2" s="41"/>
+      <c r="AB2" s="41"/>
+      <c r="AC2" s="34"/>
+      <c r="AD2" s="34"/>
+      <c r="AE2" s="34"/>
+      <c r="AF2" s="34"/>
+      <c r="AG2" s="34"/>
+      <c r="AH2" s="35"/>
+      <c r="AI2" s="35"/>
     </row>
     <row r="3" spans="1:35" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
@@ -4538,18 +4543,6 @@
     </row>
   </sheetData>
   <mergeCells count="28">
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="B1:B2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="D1:I1"/>
-    <mergeCell ref="D2:E2"/>
-    <mergeCell ref="F2:G2"/>
-    <mergeCell ref="H2:I2"/>
-    <mergeCell ref="K1:M1"/>
-    <mergeCell ref="N1:N2"/>
-    <mergeCell ref="O1:O2"/>
-    <mergeCell ref="P1:P2"/>
-    <mergeCell ref="Q1:Q2"/>
     <mergeCell ref="R1:R2"/>
     <mergeCell ref="AG1:AG2"/>
     <mergeCell ref="AH1:AH2"/>
@@ -4566,6 +4559,18 @@
     <mergeCell ref="AB1:AB2"/>
     <mergeCell ref="AC1:AE2"/>
     <mergeCell ref="AF1:AF2"/>
+    <mergeCell ref="K1:M1"/>
+    <mergeCell ref="N1:N2"/>
+    <mergeCell ref="O1:O2"/>
+    <mergeCell ref="P1:P2"/>
+    <mergeCell ref="Q1:Q2"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="D1:I1"/>
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="F2:G2"/>
+    <mergeCell ref="H2:I2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>

</xml_diff>